<commit_message>
state: bot run 2026-09-05T04:26 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_us.xlsx
+++ b/data/trade_log_us.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2552,6 +2552,694 @@
       <c r="K49" t="inlineStr">
         <is>
           <t>BELOW_BAND (Close 169.96 &lt;= Upper 170.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>230.36</v>
+      </c>
+      <c r="E50" t="n">
+        <v>232.35</v>
+      </c>
+      <c r="F50" t="n">
+        <v>232.35</v>
+      </c>
+      <c r="G50" t="n">
+        <v>222.89</v>
+      </c>
+      <c r="H50" t="n">
+        <v>219.04</v>
+      </c>
+      <c r="I50" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 230.36 &lt;= Upper 232.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>354.08</v>
+      </c>
+      <c r="E51" t="n">
+        <v>373.23</v>
+      </c>
+      <c r="F51" t="n">
+        <v>373.23</v>
+      </c>
+      <c r="G51" t="n">
+        <v>357.35</v>
+      </c>
+      <c r="H51" t="n">
+        <v>351.67</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J51" t="b">
+        <v>0</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 354.08 &lt;= Upper 373.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>319.97</v>
+      </c>
+      <c r="E52" t="n">
+        <v>328.06</v>
+      </c>
+      <c r="F52" t="n">
+        <v>328.06</v>
+      </c>
+      <c r="G52" t="n">
+        <v>319.98</v>
+      </c>
+      <c r="H52" t="n">
+        <v>316.73</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J52" t="b">
+        <v>0</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 319.97 &lt;= Upper 328.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>499.7</v>
+      </c>
+      <c r="E53" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="F53" t="n">
+        <v>516.08</v>
+      </c>
+      <c r="G53" t="n">
+        <v>500.48</v>
+      </c>
+      <c r="H53" t="n">
+        <v>488.68</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J53" t="b">
+        <v>0</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 499.70 &lt;= Upper 516.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>616.77</v>
+      </c>
+      <c r="E54" t="n">
+        <v>619.29</v>
+      </c>
+      <c r="F54" t="n">
+        <v>619.29</v>
+      </c>
+      <c r="G54" t="n">
+        <v>589.64</v>
+      </c>
+      <c r="H54" t="n">
+        <v>583.6</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J54" t="b">
+        <v>0</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 616.77 &lt;= Upper 619.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>258.51</v>
+      </c>
+      <c r="E55" t="n">
+        <v>273.63</v>
+      </c>
+      <c r="F55" t="n">
+        <v>273.63</v>
+      </c>
+      <c r="G55" t="n">
+        <v>258.96</v>
+      </c>
+      <c r="H55" t="n">
+        <v>259.54</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J55" t="b">
+        <v>0</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 258.96 &lt;= EMA21 259.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>338.46</v>
+      </c>
+      <c r="E56" t="n">
+        <v>353.14</v>
+      </c>
+      <c r="F56" t="n">
+        <v>353.14</v>
+      </c>
+      <c r="G56" t="n">
+        <v>340.75</v>
+      </c>
+      <c r="H56" t="n">
+        <v>343.59</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J56" t="b">
+        <v>0</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 340.75 &lt;= EMA21 343.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>477.57</v>
+      </c>
+      <c r="E57" t="n">
+        <v>505.22</v>
+      </c>
+      <c r="F57" t="n">
+        <v>505.22</v>
+      </c>
+      <c r="G57" t="n">
+        <v>468.28</v>
+      </c>
+      <c r="H57" t="n">
+        <v>475.5</v>
+      </c>
+      <c r="I57" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J57" t="b">
+        <v>0</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 468.28 &lt;= EMA21 475.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>78.25</v>
+      </c>
+      <c r="E58" t="n">
+        <v>84.38</v>
+      </c>
+      <c r="F58" t="n">
+        <v>84.38</v>
+      </c>
+      <c r="G58" t="n">
+        <v>80.62</v>
+      </c>
+      <c r="H58" t="n">
+        <v>79.13</v>
+      </c>
+      <c r="I58" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J58" t="b">
+        <v>0</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 78.25 &lt;= Upper 84.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>174.33</v>
+      </c>
+      <c r="E59" t="n">
+        <v>187.21</v>
+      </c>
+      <c r="F59" t="n">
+        <v>187.21</v>
+      </c>
+      <c r="G59" t="n">
+        <v>177.88</v>
+      </c>
+      <c r="H59" t="n">
+        <v>171.96</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J59" t="b">
+        <v>0</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 174.33 &lt;= Upper 187.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>357.89</v>
+      </c>
+      <c r="E60" t="n">
+        <v>424.09</v>
+      </c>
+      <c r="F60" t="n">
+        <v>424.09</v>
+      </c>
+      <c r="G60" t="n">
+        <v>365.27</v>
+      </c>
+      <c r="H60" t="n">
+        <v>374.12</v>
+      </c>
+      <c r="I60" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="J60" t="b">
+        <v>0</v>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.27 &lt;= EMA21 374.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>184.64</v>
+      </c>
+      <c r="E61" t="n">
+        <v>204.15</v>
+      </c>
+      <c r="F61" t="n">
+        <v>204.15</v>
+      </c>
+      <c r="G61" t="n">
+        <v>181.51</v>
+      </c>
+      <c r="H61" t="n">
+        <v>173.86</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J61" t="b">
+        <v>0</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 184.64 &lt;= Upper 204.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>252.09</v>
+      </c>
+      <c r="E62" t="n">
+        <v>282.59</v>
+      </c>
+      <c r="F62" t="n">
+        <v>282.59</v>
+      </c>
+      <c r="G62" t="n">
+        <v>244.99</v>
+      </c>
+      <c r="H62" t="n">
+        <v>252.3</v>
+      </c>
+      <c r="I62" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J62" t="b">
+        <v>0</v>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 244.99 &lt;= EMA21 252.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>UBER</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>75.76000000000001</v>
+      </c>
+      <c r="E63" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="F63" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="G63" t="n">
+        <v>76.54000000000001</v>
+      </c>
+      <c r="H63" t="n">
+        <v>76.11</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J63" t="b">
+        <v>0</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 75.76 &lt;= Upper 80.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>39.59</v>
+      </c>
+      <c r="E64" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="F64" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="G64" t="n">
+        <v>37.67</v>
+      </c>
+      <c r="H64" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J64" t="b">
+        <v>0</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 39.59 &lt;= Upper 41.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>168.74</v>
+      </c>
+      <c r="E65" t="n">
+        <v>170.32</v>
+      </c>
+      <c r="F65" t="n">
+        <v>170.32</v>
+      </c>
+      <c r="G65" t="n">
+        <v>166.2</v>
+      </c>
+      <c r="H65" t="n">
+        <v>164.92</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J65" t="b">
+        <v>0</v>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 168.74 &lt;= Upper 170.32)</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3368,6 +4056,39 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>04:26:39</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>9828.719999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-171.28</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>